<commit_message>
cleaning process no relevant changes, data_data_processing chiara funzioni per pulizia dati funzionanti tranne età con anno di nascita da sistemare
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_7DD945CF15660E0F62355476585DCE3A8742D602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B768188C-54F6-4860-AE59-1D44E00C6C65}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_7DD945CF15660E0F62355476585DCE3A8742D602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16647D70-D90C-4449-9EEE-EAE032D8937D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-3705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1962,6 +1975,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1989,20 +2016,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2021,11 +2034,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}" name="Tabella1" displayName="Tabella1" ref="A1:K487" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}" name="Tabella1" displayName="Tabella1" ref="A1:K487" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:K487" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}">
-    <filterColumn colId="2">
+    <filterColumn colId="1">
       <filters>
-        <filter val="visit"/>
+        <filter val="BLCHANGE"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2333,6 +2346,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K487"/>
   <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="8" width="0" hidden="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -2465,7 +2481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2497,7 +2513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -3300,7 +3316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -3844,7 +3860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>121</v>
       </c>
@@ -3876,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>121</v>
       </c>
@@ -4077,7 +4093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>121</v>
       </c>
@@ -4306,7 +4322,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>154</v>
       </c>
@@ -4390,7 +4406,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>154</v>
       </c>
@@ -4586,7 +4602,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>154</v>
       </c>
@@ -4642,7 +4658,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>154</v>
       </c>
@@ -4656,7 +4672,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>154</v>
       </c>
@@ -4754,7 +4770,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>154</v>
       </c>
@@ -4768,7 +4784,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>154</v>
       </c>
@@ -4894,7 +4910,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>154</v>
       </c>
@@ -9084,7 +9100,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="406" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A406" t="s">
         <v>501</v>
       </c>
@@ -9113,7 +9129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="407" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A407" t="s">
         <v>501</v>
       </c>
@@ -9142,7 +9158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="408" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A408" t="s">
         <v>501</v>
       </c>
@@ -9258,7 +9274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="412" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A412" t="s">
         <v>501</v>
       </c>
@@ -9293,7 +9309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="413" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A413" t="s">
         <v>501</v>
       </c>
@@ -9325,7 +9341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="414" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A414" t="s">
         <v>501</v>
       </c>
@@ -9357,7 +9373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="415" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A415" t="s">
         <v>501</v>
       </c>
@@ -9389,7 +9405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="416" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A416" t="s">
         <v>501</v>
       </c>
@@ -9421,7 +9437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="417" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A417" t="s">
         <v>501</v>
       </c>
@@ -9453,7 +9469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="418" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A418" t="s">
         <v>501</v>
       </c>
@@ -9485,7 +9501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="419" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A419" t="s">
         <v>501</v>
       </c>
@@ -9517,7 +9533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="420" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A420" t="s">
         <v>501</v>
       </c>
@@ -9549,7 +9565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="421" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A421" t="s">
         <v>501</v>
       </c>
@@ -9581,7 +9597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="422" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A422" t="s">
         <v>501</v>
       </c>
@@ -9613,7 +9629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="423" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A423" t="s">
         <v>501</v>
       </c>
@@ -9729,7 +9745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="427" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>529</v>
       </c>
@@ -9758,7 +9774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="428" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>529</v>
       </c>
@@ -9772,7 +9788,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="429" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>529</v>
       </c>
@@ -10045,7 +10061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="438" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>548</v>
       </c>
@@ -10353,7 +10369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="448" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>564</v>
       </c>
@@ -10382,7 +10398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="449" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>564</v>
       </c>
@@ -10396,7 +10412,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="450" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>564</v>
       </c>
@@ -10483,7 +10499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="453" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>564</v>
       </c>
@@ -10608,7 +10624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="457" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
         <v>570</v>
       </c>
@@ -10640,7 +10656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="458" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
         <v>570</v>
       </c>
@@ -11470,7 +11486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="483" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
         <v>570</v>
       </c>

</xml_diff>

<commit_message>
Risoluzione problema conto età da anni, commento funzioni e alcuni miglioramenti ATTENZIONE rifare un check perchè funzioni tutto
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_7DD945CF15660E0F62355476585DCE3A8742D602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16647D70-D90C-4449-9EEE-EAE032D8937D}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="11_7DD945CF15660E0F62355476585DCE3A8742D602" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F8174E-5949-4130-A936-60B80E04022D}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-3705" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2035,13 +2035,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}" name="Tabella1" displayName="Tabella1" ref="A1:K487" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A1:K487" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="BLCHANGE"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K487" xr:uid="{E63766A8-0837-4848-AAF2-CB2948CF75CA}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{2DD95BA9-1A58-4558-BABE-1BC136183262}" name="file_name"/>
     <tableColumn id="2" xr3:uid="{DD74AB91-ABD2-432A-9E15-61C6BEBC4616}" name="file_code"/>
@@ -2347,7 +2341,11 @@
   <dimension ref="A1:K487"/>
   <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="8" width="0" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="76.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -2385,7 +2383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2417,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2449,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -2481,7 +2479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2513,7 +2511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2545,7 +2543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2577,7 +2575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2609,7 +2607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -2641,7 +2639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2673,7 +2671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2705,7 +2703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2737,7 +2735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2772,7 +2770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -2804,7 +2802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -2836,7 +2834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -2868,7 +2866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -2900,7 +2898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -2932,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -2964,7 +2962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -2996,7 +2994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -3028,7 +3026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -3060,7 +3058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -3092,7 +3090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -3124,7 +3122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -3156,7 +3154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -3188,7 +3186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -3220,7 +3218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -3252,7 +3250,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -3284,7 +3282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -3316,7 +3314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -3348,7 +3346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -3380,7 +3378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -3412,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -3444,7 +3442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -3476,7 +3474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -3508,7 +3506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -3540,7 +3538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -3572,7 +3570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -3604,7 +3602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -3636,7 +3634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -3668,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>11</v>
       </c>
@@ -3700,7 +3698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>11</v>
       </c>
@@ -3732,7 +3730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -3764,7 +3762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>11</v>
       </c>
@@ -3796,7 +3794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>121</v>
       </c>
@@ -3828,7 +3826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>121</v>
       </c>
@@ -3860,7 +3858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>121</v>
       </c>
@@ -3892,7 +3890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>121</v>
       </c>
@@ -3924,7 +3922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>121</v>
       </c>
@@ -3956,7 +3954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>121</v>
       </c>
@@ -3991,7 +3989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>121</v>
       </c>
@@ -4026,7 +4024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>121</v>
       </c>
@@ -4061,7 +4059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>121</v>
       </c>
@@ -4093,7 +4091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>121</v>
       </c>
@@ -4125,7 +4123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -4139,7 +4137,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>121</v>
       </c>
@@ -4153,7 +4151,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>121</v>
       </c>
@@ -4167,7 +4165,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>121</v>
       </c>
@@ -4181,7 +4179,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>121</v>
       </c>
@@ -4213,7 +4211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>121</v>
       </c>
@@ -4227,7 +4225,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>121</v>
       </c>
@@ -4262,7 +4260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>121</v>
       </c>
@@ -4294,7 +4292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>121</v>
       </c>
@@ -4308,7 +4306,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>154</v>
       </c>
@@ -4322,7 +4320,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>154</v>
       </c>
@@ -4336,7 +4334,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>154</v>
       </c>
@@ -4350,7 +4348,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>154</v>
       </c>
@@ -4364,7 +4362,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>154</v>
       </c>
@@ -4378,7 +4376,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>154</v>
       </c>
@@ -4392,7 +4390,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>154</v>
       </c>
@@ -4406,7 +4404,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>154</v>
       </c>
@@ -4420,7 +4418,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>154</v>
       </c>
@@ -4434,7 +4432,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>154</v>
       </c>
@@ -4448,7 +4446,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -4462,7 +4460,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>154</v>
       </c>
@@ -4476,7 +4474,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>154</v>
       </c>
@@ -4490,7 +4488,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>154</v>
       </c>
@@ -4504,7 +4502,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>154</v>
       </c>
@@ -4518,7 +4516,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>154</v>
       </c>
@@ -4532,7 +4530,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>154</v>
       </c>
@@ -4546,7 +4544,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>154</v>
       </c>
@@ -4560,7 +4558,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>154</v>
       </c>
@@ -4574,7 +4572,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>154</v>
       </c>
@@ -4588,7 +4586,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>154</v>
       </c>
@@ -4602,7 +4600,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>154</v>
       </c>
@@ -4616,7 +4614,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -4630,7 +4628,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>154</v>
       </c>
@@ -4644,7 +4642,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>154</v>
       </c>
@@ -4658,7 +4656,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>154</v>
       </c>
@@ -4672,7 +4670,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>154</v>
       </c>
@@ -4686,7 +4684,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>154</v>
       </c>
@@ -4700,7 +4698,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>154</v>
       </c>
@@ -4714,7 +4712,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>154</v>
       </c>
@@ -4728,7 +4726,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>154</v>
       </c>
@@ -4742,7 +4740,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>154</v>
       </c>
@@ -4756,7 +4754,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="97" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>154</v>
       </c>
@@ -4770,7 +4768,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="98" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>154</v>
       </c>
@@ -4784,7 +4782,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="99" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>154</v>
       </c>
@@ -4798,7 +4796,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="100" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>154</v>
       </c>
@@ -4812,7 +4810,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="101" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>154</v>
       </c>
@@ -4826,7 +4824,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="102" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>154</v>
       </c>
@@ -4840,7 +4838,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="103" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>154</v>
       </c>
@@ -4854,7 +4852,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="104" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>154</v>
       </c>
@@ -4868,7 +4866,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="105" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>154</v>
       </c>
@@ -4882,7 +4880,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="106" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>154</v>
       </c>
@@ -4896,7 +4894,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="107" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>154</v>
       </c>
@@ -4910,7 +4908,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="108" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>154</v>
       </c>
@@ -4924,7 +4922,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="109" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>199</v>
       </c>
@@ -4956,7 +4954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>199</v>
       </c>
@@ -4970,7 +4968,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="111" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>199</v>
       </c>
@@ -4984,7 +4982,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="112" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>199</v>
       </c>
@@ -4998,7 +4996,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>199</v>
       </c>
@@ -5012,7 +5010,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>199</v>
       </c>
@@ -5026,7 +5024,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>199</v>
       </c>
@@ -5040,7 +5038,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>199</v>
       </c>
@@ -5054,7 +5052,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>199</v>
       </c>
@@ -5068,7 +5066,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>199</v>
       </c>
@@ -5082,7 +5080,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>199</v>
       </c>
@@ -5096,7 +5094,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>199</v>
       </c>
@@ -5110,7 +5108,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>199</v>
       </c>
@@ -5124,7 +5122,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>199</v>
       </c>
@@ -5138,7 +5136,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>199</v>
       </c>
@@ -5152,7 +5150,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>199</v>
       </c>
@@ -5166,7 +5164,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>199</v>
       </c>
@@ -5180,7 +5178,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>199</v>
       </c>
@@ -5194,7 +5192,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>199</v>
       </c>
@@ -5208,7 +5206,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>199</v>
       </c>
@@ -5222,7 +5220,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>199</v>
       </c>
@@ -5236,7 +5234,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>199</v>
       </c>
@@ -5250,7 +5248,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>199</v>
       </c>
@@ -5264,7 +5262,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>199</v>
       </c>
@@ -5278,7 +5276,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>199</v>
       </c>
@@ -5292,7 +5290,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>199</v>
       </c>
@@ -5306,7 +5304,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>199</v>
       </c>
@@ -5320,7 +5318,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>199</v>
       </c>
@@ -5334,7 +5332,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="137" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>199</v>
       </c>
@@ -5348,7 +5346,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>199</v>
       </c>
@@ -5362,7 +5360,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>199</v>
       </c>
@@ -5376,7 +5374,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>199</v>
       </c>
@@ -5390,7 +5388,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>199</v>
       </c>
@@ -5404,7 +5402,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>199</v>
       </c>
@@ -5418,7 +5416,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="143" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>199</v>
       </c>
@@ -5432,7 +5430,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>199</v>
       </c>
@@ -5446,7 +5444,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>199</v>
       </c>
@@ -5460,7 +5458,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>199</v>
       </c>
@@ -5474,7 +5472,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>199</v>
       </c>
@@ -5488,7 +5486,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>199</v>
       </c>
@@ -5502,7 +5500,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>199</v>
       </c>
@@ -5516,7 +5514,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="150" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>199</v>
       </c>
@@ -5530,7 +5528,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="151" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>199</v>
       </c>
@@ -5544,7 +5542,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>199</v>
       </c>
@@ -5558,7 +5556,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="153" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>199</v>
       </c>
@@ -5572,7 +5570,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>199</v>
       </c>
@@ -5586,7 +5584,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>199</v>
       </c>
@@ -5600,7 +5598,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>199</v>
       </c>
@@ -5614,7 +5612,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>199</v>
       </c>
@@ -5628,7 +5626,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>199</v>
       </c>
@@ -5642,7 +5640,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>199</v>
       </c>
@@ -5656,7 +5654,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>199</v>
       </c>
@@ -5670,7 +5668,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>199</v>
       </c>
@@ -5684,7 +5682,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>199</v>
       </c>
@@ -5698,7 +5696,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>199</v>
       </c>
@@ -5712,7 +5710,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>199</v>
       </c>
@@ -5726,7 +5724,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>199</v>
       </c>
@@ -5740,7 +5738,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>199</v>
       </c>
@@ -5754,7 +5752,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>199</v>
       </c>
@@ -5768,7 +5766,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>199</v>
       </c>
@@ -5782,7 +5780,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>199</v>
       </c>
@@ -5796,7 +5794,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>199</v>
       </c>
@@ -5810,7 +5808,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>199</v>
       </c>
@@ -5824,7 +5822,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>199</v>
       </c>
@@ -5838,7 +5836,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>199</v>
       </c>
@@ -5852,7 +5850,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>199</v>
       </c>
@@ -5866,7 +5864,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>199</v>
       </c>
@@ -5880,7 +5878,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>199</v>
       </c>
@@ -5894,7 +5892,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>199</v>
       </c>
@@ -5908,7 +5906,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>199</v>
       </c>
@@ -5922,7 +5920,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>199</v>
       </c>
@@ -5936,7 +5934,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>199</v>
       </c>
@@ -5950,7 +5948,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>199</v>
       </c>
@@ -5964,7 +5962,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>199</v>
       </c>
@@ -5978,7 +5976,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>199</v>
       </c>
@@ -5992,7 +5990,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>199</v>
       </c>
@@ -6006,7 +6004,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>199</v>
       </c>
@@ -6020,7 +6018,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>199</v>
       </c>
@@ -6034,7 +6032,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>199</v>
       </c>
@@ -6048,7 +6046,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>199</v>
       </c>
@@ -6062,7 +6060,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>199</v>
       </c>
@@ -6076,7 +6074,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>199</v>
       </c>
@@ -6090,7 +6088,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>199</v>
       </c>
@@ -6104,7 +6102,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>199</v>
       </c>
@@ -6118,7 +6116,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>199</v>
       </c>
@@ -6132,7 +6130,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>199</v>
       </c>
@@ -6146,7 +6144,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>199</v>
       </c>
@@ -6160,7 +6158,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>199</v>
       </c>
@@ -6174,7 +6172,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>199</v>
       </c>
@@ -6188,7 +6186,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>199</v>
       </c>
@@ -6202,7 +6200,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>199</v>
       </c>
@@ -6216,7 +6214,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>199</v>
       </c>
@@ -6230,7 +6228,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>199</v>
       </c>
@@ -6244,7 +6242,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="202" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>199</v>
       </c>
@@ -6258,7 +6256,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>199</v>
       </c>
@@ -6272,7 +6270,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="204" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>199</v>
       </c>
@@ -6286,7 +6284,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="205" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>199</v>
       </c>
@@ -6300,7 +6298,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="206" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>199</v>
       </c>
@@ -6314,7 +6312,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="207" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>199</v>
       </c>
@@ -6328,7 +6326,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="208" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>199</v>
       </c>
@@ -6342,7 +6340,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="209" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>199</v>
       </c>
@@ -6356,7 +6354,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="210" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>199</v>
       </c>
@@ -6370,7 +6368,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="211" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>199</v>
       </c>
@@ -6384,7 +6382,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="212" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>199</v>
       </c>
@@ -6398,7 +6396,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="213" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>199</v>
       </c>
@@ -6412,7 +6410,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="214" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>199</v>
       </c>
@@ -6426,7 +6424,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="215" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>199</v>
       </c>
@@ -6440,7 +6438,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="216" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>199</v>
       </c>
@@ -6454,7 +6452,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="217" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>199</v>
       </c>
@@ -6468,7 +6466,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="218" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>199</v>
       </c>
@@ -6482,7 +6480,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="219" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>199</v>
       </c>
@@ -6496,7 +6494,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="220" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>199</v>
       </c>
@@ -6510,7 +6508,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="221" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>199</v>
       </c>
@@ -6524,7 +6522,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="222" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>199</v>
       </c>
@@ -6538,7 +6536,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="223" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>199</v>
       </c>
@@ -6552,7 +6550,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="224" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>199</v>
       </c>
@@ -6566,7 +6564,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="225" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>199</v>
       </c>
@@ -6580,7 +6578,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="226" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>199</v>
       </c>
@@ -6594,7 +6592,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="227" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>199</v>
       </c>
@@ -6608,7 +6606,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="228" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>199</v>
       </c>
@@ -6622,7 +6620,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="229" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>199</v>
       </c>
@@ -6636,7 +6634,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="230" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>199</v>
       </c>
@@ -6650,7 +6648,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="231" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>199</v>
       </c>
@@ -6664,7 +6662,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="232" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>199</v>
       </c>
@@ -6678,7 +6676,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="233" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>199</v>
       </c>
@@ -6692,7 +6690,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="234" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>199</v>
       </c>
@@ -6706,7 +6704,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="235" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>199</v>
       </c>
@@ -6720,7 +6718,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="236" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>199</v>
       </c>
@@ -6734,7 +6732,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="237" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>199</v>
       </c>
@@ -6748,7 +6746,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="238" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>199</v>
       </c>
@@ -6762,7 +6760,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="239" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>199</v>
       </c>
@@ -6776,7 +6774,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="240" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>199</v>
       </c>
@@ -6790,7 +6788,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="241" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>199</v>
       </c>
@@ -6804,7 +6802,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="242" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>199</v>
       </c>
@@ -6818,7 +6816,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="243" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>199</v>
       </c>
@@ -6832,7 +6830,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="244" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>199</v>
       </c>
@@ -6846,7 +6844,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="245" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>199</v>
       </c>
@@ -6860,7 +6858,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="246" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>199</v>
       </c>
@@ -6874,7 +6872,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="247" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>199</v>
       </c>
@@ -6888,7 +6886,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="248" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>199</v>
       </c>
@@ -6902,7 +6900,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="249" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>199</v>
       </c>
@@ -6916,7 +6914,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="250" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>199</v>
       </c>
@@ -6930,7 +6928,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="251" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>199</v>
       </c>
@@ -6944,7 +6942,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="252" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>199</v>
       </c>
@@ -6958,7 +6956,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="253" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>199</v>
       </c>
@@ -6972,7 +6970,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="254" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>199</v>
       </c>
@@ -6986,7 +6984,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="255" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>199</v>
       </c>
@@ -7000,7 +6998,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="256" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>199</v>
       </c>
@@ -7014,7 +7012,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="257" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>199</v>
       </c>
@@ -7028,7 +7026,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="258" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>199</v>
       </c>
@@ -7042,7 +7040,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="259" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>199</v>
       </c>
@@ -7056,7 +7054,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="260" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>199</v>
       </c>
@@ -7070,7 +7068,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="261" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>199</v>
       </c>
@@ -7084,7 +7082,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="262" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>199</v>
       </c>
@@ -7098,7 +7096,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="263" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>199</v>
       </c>
@@ -7112,7 +7110,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="264" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>199</v>
       </c>
@@ -7126,7 +7124,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="265" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>199</v>
       </c>
@@ -7140,7 +7138,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="266" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>199</v>
       </c>
@@ -7154,7 +7152,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="267" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>199</v>
       </c>
@@ -7168,7 +7166,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="268" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>199</v>
       </c>
@@ -7182,7 +7180,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="269" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>199</v>
       </c>
@@ -7196,7 +7194,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="270" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>199</v>
       </c>
@@ -7210,7 +7208,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="271" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>199</v>
       </c>
@@ -7224,7 +7222,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="272" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>199</v>
       </c>
@@ -7238,7 +7236,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="273" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>199</v>
       </c>
@@ -7252,7 +7250,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="274" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>199</v>
       </c>
@@ -7266,7 +7264,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="275" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>199</v>
       </c>
@@ -7280,7 +7278,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="276" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>199</v>
       </c>
@@ -7294,7 +7292,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="277" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>199</v>
       </c>
@@ -7308,7 +7306,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="278" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>199</v>
       </c>
@@ -7322,7 +7320,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="279" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>199</v>
       </c>
@@ -7336,7 +7334,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="280" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>199</v>
       </c>
@@ -7350,7 +7348,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="281" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>199</v>
       </c>
@@ -7364,7 +7362,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="282" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>199</v>
       </c>
@@ -7378,7 +7376,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="283" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>199</v>
       </c>
@@ -7392,7 +7390,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="284" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>199</v>
       </c>
@@ -7406,7 +7404,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="285" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>199</v>
       </c>
@@ -7420,7 +7418,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="286" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>199</v>
       </c>
@@ -7434,7 +7432,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="287" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>199</v>
       </c>
@@ -7448,7 +7446,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="288" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>199</v>
       </c>
@@ -7462,7 +7460,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="289" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>199</v>
       </c>
@@ -7476,7 +7474,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="290" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>199</v>
       </c>
@@ -7490,7 +7488,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="291" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>199</v>
       </c>
@@ -7504,7 +7502,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="292" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>199</v>
       </c>
@@ -7518,7 +7516,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="293" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>199</v>
       </c>
@@ -7532,7 +7530,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="294" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>199</v>
       </c>
@@ -7546,7 +7544,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="295" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>199</v>
       </c>
@@ -7560,7 +7558,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="296" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>199</v>
       </c>
@@ -7574,7 +7572,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="297" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>199</v>
       </c>
@@ -7588,7 +7586,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="298" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>199</v>
       </c>
@@ -7602,7 +7600,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="299" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>199</v>
       </c>
@@ -7616,7 +7614,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="300" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>199</v>
       </c>
@@ -7630,7 +7628,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="301" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>199</v>
       </c>
@@ -7644,7 +7642,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="302" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>199</v>
       </c>
@@ -7658,7 +7656,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="303" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>199</v>
       </c>
@@ -7672,7 +7670,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="304" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>199</v>
       </c>
@@ -7686,7 +7684,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="305" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>199</v>
       </c>
@@ -7700,7 +7698,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="306" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>199</v>
       </c>
@@ -7714,7 +7712,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="307" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>199</v>
       </c>
@@ -7728,7 +7726,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="308" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>199</v>
       </c>
@@ -7742,7 +7740,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="309" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>199</v>
       </c>
@@ -7756,7 +7754,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="310" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>199</v>
       </c>
@@ -7770,7 +7768,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="311" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>199</v>
       </c>
@@ -7784,7 +7782,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="312" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>199</v>
       </c>
@@ -7798,7 +7796,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="313" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>199</v>
       </c>
@@ -7812,7 +7810,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="314" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>199</v>
       </c>
@@ -7826,7 +7824,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="315" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>199</v>
       </c>
@@ -7840,7 +7838,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="316" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>199</v>
       </c>
@@ -7854,7 +7852,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="317" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>199</v>
       </c>
@@ -7868,7 +7866,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="318" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>199</v>
       </c>
@@ -7882,7 +7880,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="319" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>199</v>
       </c>
@@ -7896,7 +7894,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="320" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>199</v>
       </c>
@@ -7910,7 +7908,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="321" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>199</v>
       </c>
@@ -7924,7 +7922,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="322" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>199</v>
       </c>
@@ -7938,7 +7936,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="323" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>199</v>
       </c>
@@ -7952,7 +7950,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="324" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>199</v>
       </c>
@@ -7966,7 +7964,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="325" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>199</v>
       </c>
@@ -7980,7 +7978,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="326" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>199</v>
       </c>
@@ -7994,7 +7992,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="327" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>199</v>
       </c>
@@ -8008,7 +8006,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="328" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>199</v>
       </c>
@@ -8022,7 +8020,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="329" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>199</v>
       </c>
@@ -8036,7 +8034,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="330" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>199</v>
       </c>
@@ -8050,7 +8048,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="331" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>199</v>
       </c>
@@ -8064,7 +8062,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="332" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>199</v>
       </c>
@@ -8078,7 +8076,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="333" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>199</v>
       </c>
@@ -8092,7 +8090,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="334" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>199</v>
       </c>
@@ -8106,7 +8104,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="335" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>199</v>
       </c>
@@ -8120,7 +8118,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="336" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>199</v>
       </c>
@@ -8134,7 +8132,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="337" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>199</v>
       </c>
@@ -8148,7 +8146,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>199</v>
       </c>
@@ -8162,7 +8160,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>199</v>
       </c>
@@ -8176,7 +8174,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>199</v>
       </c>
@@ -8190,7 +8188,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>199</v>
       </c>
@@ -8204,7 +8202,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>199</v>
       </c>
@@ -8218,7 +8216,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>199</v>
       </c>
@@ -8232,7 +8230,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="344" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>199</v>
       </c>
@@ -8246,7 +8244,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>199</v>
       </c>
@@ -8260,7 +8258,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>199</v>
       </c>
@@ -8274,7 +8272,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="347" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>199</v>
       </c>
@@ -8288,7 +8286,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>199</v>
       </c>
@@ -8302,7 +8300,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>199</v>
       </c>
@@ -8316,7 +8314,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="350" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>199</v>
       </c>
@@ -8330,7 +8328,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="351" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>199</v>
       </c>
@@ -8344,7 +8342,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>199</v>
       </c>
@@ -8358,7 +8356,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="353" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>199</v>
       </c>
@@ -8372,7 +8370,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="354" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>199</v>
       </c>
@@ -8386,7 +8384,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="355" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>199</v>
       </c>
@@ -8400,7 +8398,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="356" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>199</v>
       </c>
@@ -8414,7 +8412,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="357" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>199</v>
       </c>
@@ -8428,7 +8426,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="358" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>199</v>
       </c>
@@ -8442,7 +8440,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="359" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>199</v>
       </c>
@@ -8456,7 +8454,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="360" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>199</v>
       </c>
@@ -8470,7 +8468,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="361" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>199</v>
       </c>
@@ -8484,7 +8482,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="362" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>199</v>
       </c>
@@ -8498,7 +8496,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="363" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>199</v>
       </c>
@@ -8512,7 +8510,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="364" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>199</v>
       </c>
@@ -8526,7 +8524,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="365" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>199</v>
       </c>
@@ -8540,7 +8538,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="366" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>199</v>
       </c>
@@ -8554,7 +8552,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="367" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>199</v>
       </c>
@@ -8568,7 +8566,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="368" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>199</v>
       </c>
@@ -8582,7 +8580,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="369" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>199</v>
       </c>
@@ -8596,7 +8594,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="370" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>199</v>
       </c>
@@ -8610,7 +8608,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="371" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>199</v>
       </c>
@@ -8624,7 +8622,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="372" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>199</v>
       </c>
@@ -8638,7 +8636,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="373" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>199</v>
       </c>
@@ -8652,7 +8650,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="374" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>199</v>
       </c>
@@ -8666,7 +8664,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="375" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>199</v>
       </c>
@@ -8680,7 +8678,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="376" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>199</v>
       </c>
@@ -8694,7 +8692,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="377" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>199</v>
       </c>
@@ -8708,7 +8706,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="378" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>199</v>
       </c>
@@ -8722,7 +8720,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="379" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>199</v>
       </c>
@@ -8736,7 +8734,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="380" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>199</v>
       </c>
@@ -8750,7 +8748,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="381" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>199</v>
       </c>
@@ -8764,7 +8762,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="382" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>199</v>
       </c>
@@ -8778,7 +8776,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="383" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>199</v>
       </c>
@@ -8792,7 +8790,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="384" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>199</v>
       </c>
@@ -8806,7 +8804,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="385" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>199</v>
       </c>
@@ -8820,7 +8818,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="386" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>199</v>
       </c>
@@ -8834,7 +8832,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="387" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>199</v>
       </c>
@@ -8848,7 +8846,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="388" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>199</v>
       </c>
@@ -8862,7 +8860,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="389" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>199</v>
       </c>
@@ -8876,7 +8874,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="390" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>199</v>
       </c>
@@ -8890,7 +8888,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="391" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A391" t="s">
         <v>199</v>
       </c>
@@ -8904,7 +8902,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="392" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A392" t="s">
         <v>199</v>
       </c>
@@ -8918,7 +8916,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="393" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A393" t="s">
         <v>199</v>
       </c>
@@ -8932,7 +8930,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="394" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A394" t="s">
         <v>199</v>
       </c>
@@ -8946,7 +8944,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="395" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A395" t="s">
         <v>199</v>
       </c>
@@ -8960,7 +8958,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="396" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A396" t="s">
         <v>199</v>
       </c>
@@ -8974,7 +8972,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="397" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A397" t="s">
         <v>199</v>
       </c>
@@ -8988,7 +8986,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="398" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A398" t="s">
         <v>199</v>
       </c>
@@ -9002,7 +9000,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="399" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A399" t="s">
         <v>199</v>
       </c>
@@ -9016,7 +9014,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="400" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A400" t="s">
         <v>199</v>
       </c>
@@ -9030,7 +9028,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="401" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A401" t="s">
         <v>199</v>
       </c>
@@ -9044,7 +9042,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="402" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A402" t="s">
         <v>199</v>
       </c>
@@ -9058,7 +9056,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="403" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A403" t="s">
         <v>199</v>
       </c>
@@ -9072,7 +9070,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="404" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A404" t="s">
         <v>199</v>
       </c>
@@ -9086,7 +9084,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="405" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A405" t="s">
         <v>199</v>
       </c>
@@ -9658,7 +9656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="424" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A424" t="s">
         <v>529</v>
       </c>
@@ -9687,7 +9685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="425" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A425" t="s">
         <v>529</v>
       </c>
@@ -9716,7 +9714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="426" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A426" t="s">
         <v>529</v>
       </c>
@@ -9745,7 +9743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="427" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A427" t="s">
         <v>529</v>
       </c>
@@ -9774,7 +9772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="428" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A428" t="s">
         <v>529</v>
       </c>
@@ -9788,7 +9786,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="429" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A429" t="s">
         <v>529</v>
       </c>
@@ -9817,7 +9815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="430" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A430" t="s">
         <v>529</v>
       </c>
@@ -9849,7 +9847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="431" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A431" t="s">
         <v>529</v>
       </c>
@@ -9878,7 +9876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="432" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A432" t="s">
         <v>529</v>
       </c>
@@ -9910,7 +9908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="433" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A433" t="s">
         <v>529</v>
       </c>
@@ -9939,7 +9937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="434" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A434" t="s">
         <v>529</v>
       </c>
@@ -9971,7 +9969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="435" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A435" t="s">
         <v>529</v>
       </c>
@@ -10003,7 +10001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="436" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A436" t="s">
         <v>529</v>
       </c>
@@ -10032,7 +10030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="437" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A437" t="s">
         <v>529</v>
       </c>
@@ -10061,7 +10059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="438" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A438" t="s">
         <v>548</v>
       </c>
@@ -10090,7 +10088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="439" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A439" t="s">
         <v>548</v>
       </c>
@@ -10119,7 +10117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="440" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A440" t="s">
         <v>548</v>
       </c>
@@ -10151,7 +10149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="441" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A441" t="s">
         <v>548</v>
       </c>
@@ -10183,7 +10181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="442" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A442" t="s">
         <v>548</v>
       </c>
@@ -10215,7 +10213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="443" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A443" t="s">
         <v>548</v>
       </c>
@@ -10247,7 +10245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="444" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A444" t="s">
         <v>548</v>
       </c>
@@ -10282,7 +10280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="445" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A445" t="s">
         <v>564</v>
       </c>
@@ -10311,7 +10309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="446" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A446" t="s">
         <v>564</v>
       </c>
@@ -10340,7 +10338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="447" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A447" t="s">
         <v>564</v>
       </c>
@@ -10369,7 +10367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="448" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A448" t="s">
         <v>564</v>
       </c>
@@ -10398,7 +10396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="449" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A449" t="s">
         <v>564</v>
       </c>
@@ -10412,7 +10410,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="450" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A450" t="s">
         <v>564</v>
       </c>
@@ -10441,7 +10439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="451" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A451" t="s">
         <v>564</v>
       </c>
@@ -10470,7 +10468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="452" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A452" t="s">
         <v>564</v>
       </c>
@@ -10499,7 +10497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="453" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A453" t="s">
         <v>564</v>
       </c>
@@ -10528,7 +10526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="454" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A454" t="s">
         <v>570</v>
       </c>
@@ -10560,7 +10558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="455" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A455" t="s">
         <v>570</v>
       </c>
@@ -10592,7 +10590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="456" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A456" t="s">
         <v>570</v>
       </c>
@@ -10624,7 +10622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="457" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A457" t="s">
         <v>570</v>
       </c>
@@ -10656,7 +10654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="458" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A458" t="s">
         <v>570</v>
       </c>
@@ -10688,7 +10686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="459" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A459" t="s">
         <v>570</v>
       </c>
@@ -10723,7 +10721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="460" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A460" t="s">
         <v>570</v>
       </c>
@@ -10758,7 +10756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="461" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A461" t="s">
         <v>570</v>
       </c>
@@ -10793,7 +10791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="462" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A462" t="s">
         <v>570</v>
       </c>
@@ -10825,7 +10823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="463" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A463" t="s">
         <v>570</v>
       </c>
@@ -10857,7 +10855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="464" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A464" t="s">
         <v>570</v>
       </c>
@@ -10889,7 +10887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="465" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A465" t="s">
         <v>570</v>
       </c>
@@ -10921,7 +10919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="466" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A466" t="s">
         <v>570</v>
       </c>
@@ -10953,7 +10951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="467" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A467" t="s">
         <v>570</v>
       </c>
@@ -10985,7 +10983,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="468" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A468" t="s">
         <v>570</v>
       </c>
@@ -11017,7 +11015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="469" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A469" t="s">
         <v>570</v>
       </c>
@@ -11049,7 +11047,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="470" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A470" t="s">
         <v>570</v>
       </c>
@@ -11081,7 +11079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="471" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A471" t="s">
         <v>570</v>
       </c>
@@ -11116,7 +11114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="472" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A472" t="s">
         <v>570</v>
       </c>
@@ -11148,7 +11146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="473" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A473" t="s">
         <v>570</v>
       </c>
@@ -11183,7 +11181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="474" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A474" t="s">
         <v>570</v>
       </c>
@@ -11215,7 +11213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="475" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A475" t="s">
         <v>570</v>
       </c>
@@ -11247,7 +11245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="476" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A476" t="s">
         <v>570</v>
       </c>
@@ -11282,7 +11280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="477" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A477" t="s">
         <v>570</v>
       </c>
@@ -11317,7 +11315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="478" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A478" t="s">
         <v>570</v>
       </c>
@@ -11352,7 +11350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="479" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A479" t="s">
         <v>570</v>
       </c>
@@ -11387,7 +11385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="480" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A480" t="s">
         <v>570</v>
       </c>
@@ -11419,7 +11417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="481" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A481" t="s">
         <v>570</v>
       </c>
@@ -11454,7 +11452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="482" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A482" t="s">
         <v>570</v>
       </c>
@@ -11486,7 +11484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="483" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A483" t="s">
         <v>570</v>
       </c>
@@ -11518,7 +11516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="484" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A484" t="s">
         <v>570</v>
       </c>
@@ -11550,7 +11548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="485" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A485" t="s">
         <v>570</v>
       </c>
@@ -11585,7 +11583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="486" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A486" t="s">
         <v>570</v>
       </c>
@@ -11620,7 +11618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="487" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A487" t="s">
         <v>570</v>
       </c>

</xml_diff>

<commit_message>
Aggirnamenti ma ancora con qualche problemino, soprattutto colonna del excel e non funziona il trasformatore in % dei volumi
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="30" documentId="11_5D050337D547D00E62355476585DCE3A87458E14" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F816B01F-9C9D-4136-9E3A-475D3756E9D2}"/>
   <bookViews>
-    <workbookView xWindow="-36480" yWindow="-4440" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35085" yWindow="-270" windowWidth="28800" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1286,6 +1286,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Variavioni varie più aggiornamento prove download
</commit_message>
<xml_diff>
--- a/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
+++ b/WP-2/Data_cleaning/ADNI_variables_statistics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ifabfoundation-my.sharepoint.com/personal/chiara_pollicini_ifabfoundation_org/Documents/Documenti/Github/AIND/WP-2/Data_cleaning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_5B1506075248620F62355476585DCE3A8744B733" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_6279E79C1467360E62355476585DCE3A8744AE35" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48652264-5DC5-468F-9C8E-FAA47753F7D0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2699" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2889" uniqueCount="511">
   <si>
     <t>file_name</t>
   </si>
@@ -1279,49 +1279,148 @@
     <t>UCSDVOL</t>
   </si>
   <si>
+    <t>sc, m06, m12, m24, m18, m36</t>
+  </si>
+  <si>
+    <t>QCPASS</t>
+  </si>
+  <si>
+    <t>1, 0</t>
+  </si>
+  <si>
+    <t>1.0, 0.0</t>
+  </si>
+  <si>
+    <t>BRAIN</t>
+  </si>
+  <si>
+    <t>1361820.0, 629016.0</t>
+  </si>
+  <si>
+    <t>EICV</t>
+  </si>
+  <si>
+    <t>1951440.0, 1059560.0</t>
+  </si>
+  <si>
+    <t>VENTRICLES</t>
+  </si>
+  <si>
+    <t>168830.0, 7552.46</t>
+  </si>
+  <si>
+    <t>LHIPPOC</t>
+  </si>
+  <si>
+    <t>5514.94, 1287.93</t>
+  </si>
+  <si>
+    <t>RHIPPOC</t>
+  </si>
+  <si>
+    <t>5750.4, 569.549</t>
+  </si>
+  <si>
+    <t>UPENN - ADNI/DIAN Study CSF Elecsys Results [ADNI1,GO,2]</t>
+  </si>
+  <si>
+    <t>UPENNBIOMK_ADNIDIAN_ES_2017</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
-    <t>sc, m06, m12, m24, m18, m36</t>
-  </si>
-  <si>
-    <t>QCPASS</t>
-  </si>
-  <si>
-    <t>1, 0</t>
-  </si>
-  <si>
-    <t>1.0, 0.0</t>
-  </si>
-  <si>
-    <t>BRAIN</t>
-  </si>
-  <si>
-    <t>1361820.0, 629016.0</t>
-  </si>
-  <si>
-    <t>EICV</t>
-  </si>
-  <si>
-    <t>1951440.0, 1059560.0</t>
-  </si>
-  <si>
-    <t>VENTRICLES</t>
-  </si>
-  <si>
-    <t>168830.0, 7552.46</t>
-  </si>
-  <si>
-    <t>LHIPPOC</t>
-  </si>
-  <si>
-    <t>5514.94, 1287.93</t>
-  </si>
-  <si>
-    <t>RHIPPOC</t>
-  </si>
-  <si>
-    <t>5750.4, 569.549</t>
+    <t>5285.0, 42.0</t>
+  </si>
+  <si>
+    <t>m60, m84, m108, m24, m36</t>
+  </si>
+  <si>
+    <t>2011-04-14, 2013-01-24, 2015-02-12, 2011-02-08, 2013-02-07</t>
+  </si>
+  <si>
+    <t>STUDY</t>
+  </si>
+  <si>
+    <t>ADNI</t>
+  </si>
+  <si>
+    <t>RUNDATE</t>
+  </si>
+  <si>
+    <t>2017-10-30, 2017-10-20, 2017-11-09, 2017-10-27, 2017-10-23</t>
+  </si>
+  <si>
+    <t>ABETA</t>
+  </si>
+  <si>
+    <t>pg/ml</t>
+  </si>
+  <si>
+    <t>2982.0, 238.0</t>
+  </si>
+  <si>
+    <t>AB40</t>
+  </si>
+  <si>
+    <t>37590.0, 5550.0</t>
+  </si>
+  <si>
+    <t>TAU</t>
+  </si>
+  <si>
+    <t>946.0, 110.0</t>
+  </si>
+  <si>
+    <t>PTAU</t>
+  </si>
+  <si>
+    <t>118.0, 8.0</t>
+  </si>
+  <si>
+    <t>A4240</t>
+  </si>
+  <si>
+    <t>0.1036, 0.0199</t>
+  </si>
+  <si>
+    <t>UPENN CSF Biomarkers Roche Elecsys [ADNI1,GO,2,3]</t>
+  </si>
+  <si>
+    <t>UPENNBIOMK_ROCHE_ELECSYS</t>
+  </si>
+  <si>
+    <t>7073.0, 3.0</t>
+  </si>
+  <si>
+    <t>bl, m12, m24, m48, m60</t>
+  </si>
+  <si>
+    <t>2005-09-12, 2006-09-13, 2005-11-22, 2006-11-28, 2005-09-07</t>
+  </si>
+  <si>
+    <t>ADNI1, ADNIGO, ADNI2, ADNI3</t>
+  </si>
+  <si>
+    <t>2016-12-14, 2017-01-09, 2016-11-22, 2017-01-06, 2016-11-17</t>
+  </si>
+  <si>
+    <t>ABETA40</t>
+  </si>
+  <si>
+    <t>37480.0, 841.0</t>
+  </si>
+  <si>
+    <t>ABETA42</t>
+  </si>
+  <si>
+    <t>4779.0, 203.0</t>
+  </si>
+  <si>
+    <t>1018.0, 80.08</t>
+  </si>
+  <si>
+    <t>108.5, 8.0</t>
   </si>
   <si>
     <t>The DIAN-ADNI Comparison Study</t>
@@ -1529,6 +1628,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1818,6 +1921,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N346"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="73.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -11193,9 +11300,6 @@
       <c r="F261" t="s">
         <v>23</v>
       </c>
-      <c r="G261" t="s">
-        <v>419</v>
-      </c>
       <c r="H261" t="s">
         <v>335</v>
       </c>
@@ -11229,9 +11333,6 @@
         <v>18</v>
       </c>
       <c r="G262" t="s">
-        <v>420</v>
-      </c>
-      <c r="H262" t="s">
         <v>419</v>
       </c>
       <c r="I262">
@@ -11266,9 +11367,6 @@
       <c r="G263" t="s">
         <v>337</v>
       </c>
-      <c r="H263" t="s">
-        <v>419</v>
-      </c>
       <c r="I263">
         <v>3128</v>
       </c>
@@ -11293,16 +11391,16 @@
         <v>159</v>
       </c>
       <c r="D264" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F264" t="s">
         <v>23</v>
       </c>
       <c r="G264" t="s">
+        <v>421</v>
+      </c>
+      <c r="H264" t="s">
         <v>422</v>
-      </c>
-      <c r="H264" t="s">
-        <v>423</v>
       </c>
       <c r="I264">
         <v>3128</v>
@@ -11328,7 +11426,7 @@
         <v>82</v>
       </c>
       <c r="D265" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E265" t="s">
         <v>254</v>
@@ -11336,11 +11434,8 @@
       <c r="F265" t="s">
         <v>23</v>
       </c>
-      <c r="G265" t="s">
-        <v>419</v>
-      </c>
       <c r="H265" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="I265">
         <v>3128</v>
@@ -11372,7 +11467,7 @@
         <v>82</v>
       </c>
       <c r="D266" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E266" t="s">
         <v>254</v>
@@ -11380,11 +11475,8 @@
       <c r="F266" t="s">
         <v>23</v>
       </c>
-      <c r="G266" t="s">
-        <v>419</v>
-      </c>
       <c r="H266" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I266">
         <v>3128</v>
@@ -11416,7 +11508,7 @@
         <v>82</v>
       </c>
       <c r="D267" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E267" t="s">
         <v>254</v>
@@ -11424,11 +11516,8 @@
       <c r="F267" t="s">
         <v>35</v>
       </c>
-      <c r="G267" t="s">
-        <v>419</v>
-      </c>
       <c r="H267" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="I267">
         <v>3128</v>
@@ -11460,7 +11549,7 @@
         <v>82</v>
       </c>
       <c r="D268" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="E268" t="s">
         <v>254</v>
@@ -11468,11 +11557,8 @@
       <c r="F268" t="s">
         <v>35</v>
       </c>
-      <c r="G268" t="s">
-        <v>419</v>
-      </c>
       <c r="H268" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="I268">
         <v>3128</v>
@@ -11504,7 +11590,7 @@
         <v>82</v>
       </c>
       <c r="D269" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E269" t="s">
         <v>254</v>
@@ -11512,11 +11598,8 @@
       <c r="F269" t="s">
         <v>35</v>
       </c>
-      <c r="G269" t="s">
-        <v>419</v>
-      </c>
       <c r="H269" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I269">
         <v>3128</v>
@@ -11537,12 +11620,758 @@
         <v>85</v>
       </c>
     </row>
+    <row r="270" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A270" t="s">
+        <v>433</v>
+      </c>
+      <c r="B270" t="s">
+        <v>434</v>
+      </c>
+      <c r="C270" t="s">
+        <v>16</v>
+      </c>
+      <c r="D270" t="s">
+        <v>22</v>
+      </c>
+      <c r="F270" t="s">
+        <v>23</v>
+      </c>
+      <c r="G270" t="s">
+        <v>435</v>
+      </c>
+      <c r="H270" t="s">
+        <v>436</v>
+      </c>
+      <c r="I270">
+        <v>422</v>
+      </c>
+      <c r="J270">
+        <v>0</v>
+      </c>
+      <c r="K270" t="s">
+        <v>144</v>
+      </c>
+      <c r="L270" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="271" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>433</v>
+      </c>
+      <c r="B271" t="s">
+        <v>434</v>
+      </c>
+      <c r="C271" t="s">
+        <v>106</v>
+      </c>
+      <c r="D271" t="s">
+        <v>107</v>
+      </c>
+      <c r="F271" t="s">
+        <v>18</v>
+      </c>
+      <c r="G271" t="s">
+        <v>437</v>
+      </c>
+      <c r="H271" t="s">
+        <v>435</v>
+      </c>
+      <c r="I271">
+        <v>422</v>
+      </c>
+      <c r="J271">
+        <v>0</v>
+      </c>
+      <c r="K271" t="s">
+        <v>144</v>
+      </c>
+      <c r="L271" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="272" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A272" t="s">
+        <v>433</v>
+      </c>
+      <c r="B272" t="s">
+        <v>434</v>
+      </c>
+      <c r="C272" t="s">
+        <v>106</v>
+      </c>
+      <c r="D272" t="s">
+        <v>31</v>
+      </c>
+      <c r="F272" t="s">
+        <v>18</v>
+      </c>
+      <c r="G272" t="s">
+        <v>438</v>
+      </c>
+      <c r="H272" t="s">
+        <v>435</v>
+      </c>
+      <c r="I272">
+        <v>422</v>
+      </c>
+      <c r="J272">
+        <v>0</v>
+      </c>
+      <c r="K272" t="s">
+        <v>144</v>
+      </c>
+      <c r="L272" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="273" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A273" t="s">
+        <v>433</v>
+      </c>
+      <c r="B273" t="s">
+        <v>434</v>
+      </c>
+      <c r="C273" t="s">
+        <v>25</v>
+      </c>
+      <c r="D273" t="s">
+        <v>439</v>
+      </c>
+      <c r="F273" t="s">
+        <v>18</v>
+      </c>
+      <c r="G273" t="s">
+        <v>440</v>
+      </c>
+      <c r="H273" t="s">
+        <v>435</v>
+      </c>
+      <c r="I273">
+        <v>422</v>
+      </c>
+      <c r="J273">
+        <v>0</v>
+      </c>
+      <c r="K273" t="s">
+        <v>144</v>
+      </c>
+      <c r="L273" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="274" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A274" t="s">
+        <v>433</v>
+      </c>
+      <c r="B274" t="s">
+        <v>434</v>
+      </c>
+      <c r="C274" t="s">
+        <v>106</v>
+      </c>
+      <c r="D274" t="s">
+        <v>441</v>
+      </c>
+      <c r="F274" t="s">
+        <v>18</v>
+      </c>
+      <c r="G274" t="s">
+        <v>442</v>
+      </c>
+      <c r="H274" t="s">
+        <v>435</v>
+      </c>
+      <c r="I274">
+        <v>422</v>
+      </c>
+      <c r="J274">
+        <v>0</v>
+      </c>
+      <c r="K274" t="s">
+        <v>144</v>
+      </c>
+      <c r="L274" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="275" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A275" t="s">
+        <v>433</v>
+      </c>
+      <c r="B275" t="s">
+        <v>434</v>
+      </c>
+      <c r="C275" t="s">
+        <v>56</v>
+      </c>
+      <c r="D275" t="s">
+        <v>443</v>
+      </c>
+      <c r="E275" t="s">
+        <v>444</v>
+      </c>
+      <c r="F275" t="s">
+        <v>23</v>
+      </c>
+      <c r="G275" t="s">
+        <v>435</v>
+      </c>
+      <c r="H275" t="s">
+        <v>445</v>
+      </c>
+      <c r="I275">
+        <v>422</v>
+      </c>
+      <c r="J275">
+        <v>0</v>
+      </c>
+      <c r="K275" t="s">
+        <v>144</v>
+      </c>
+      <c r="L275" t="s">
+        <v>21</v>
+      </c>
+      <c r="M275" t="s">
+        <v>61</v>
+      </c>
+      <c r="N275" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="276" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A276" t="s">
+        <v>433</v>
+      </c>
+      <c r="B276" t="s">
+        <v>434</v>
+      </c>
+      <c r="C276" t="s">
+        <v>56</v>
+      </c>
+      <c r="D276" t="s">
+        <v>446</v>
+      </c>
+      <c r="E276" t="s">
+        <v>444</v>
+      </c>
+      <c r="F276" t="s">
+        <v>23</v>
+      </c>
+      <c r="G276" t="s">
+        <v>435</v>
+      </c>
+      <c r="H276" t="s">
+        <v>447</v>
+      </c>
+      <c r="I276">
+        <v>422</v>
+      </c>
+      <c r="J276">
+        <v>0</v>
+      </c>
+      <c r="K276" t="s">
+        <v>144</v>
+      </c>
+      <c r="L276" t="s">
+        <v>21</v>
+      </c>
+      <c r="M276" t="s">
+        <v>61</v>
+      </c>
+      <c r="N276" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="277" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A277" t="s">
+        <v>433</v>
+      </c>
+      <c r="B277" t="s">
+        <v>434</v>
+      </c>
+      <c r="C277" t="s">
+        <v>120</v>
+      </c>
+      <c r="D277" t="s">
+        <v>448</v>
+      </c>
+      <c r="E277" t="s">
+        <v>444</v>
+      </c>
+      <c r="F277" t="s">
+        <v>23</v>
+      </c>
+      <c r="G277" t="s">
+        <v>435</v>
+      </c>
+      <c r="H277" t="s">
+        <v>449</v>
+      </c>
+      <c r="I277">
+        <v>422</v>
+      </c>
+      <c r="J277">
+        <v>0</v>
+      </c>
+      <c r="K277" t="s">
+        <v>144</v>
+      </c>
+      <c r="L277" t="s">
+        <v>21</v>
+      </c>
+      <c r="M277" t="s">
+        <v>61</v>
+      </c>
+      <c r="N277" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="278" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A278" t="s">
+        <v>433</v>
+      </c>
+      <c r="B278" t="s">
+        <v>434</v>
+      </c>
+      <c r="C278" t="s">
+        <v>120</v>
+      </c>
+      <c r="D278" t="s">
+        <v>450</v>
+      </c>
+      <c r="E278" t="s">
+        <v>444</v>
+      </c>
+      <c r="F278" t="s">
+        <v>35</v>
+      </c>
+      <c r="G278" t="s">
+        <v>435</v>
+      </c>
+      <c r="H278" t="s">
+        <v>451</v>
+      </c>
+      <c r="I278">
+        <v>421</v>
+      </c>
+      <c r="J278">
+        <v>1</v>
+      </c>
+      <c r="K278" t="s">
+        <v>144</v>
+      </c>
+      <c r="L278" t="s">
+        <v>21</v>
+      </c>
+      <c r="M278" t="s">
+        <v>61</v>
+      </c>
+      <c r="N278" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="279" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A279" t="s">
+        <v>433</v>
+      </c>
+      <c r="B279" t="s">
+        <v>434</v>
+      </c>
+      <c r="C279" t="s">
+        <v>56</v>
+      </c>
+      <c r="D279" t="s">
+        <v>452</v>
+      </c>
+      <c r="E279" t="s">
+        <v>444</v>
+      </c>
+      <c r="F279" t="s">
+        <v>35</v>
+      </c>
+      <c r="G279" t="s">
+        <v>435</v>
+      </c>
+      <c r="H279" t="s">
+        <v>453</v>
+      </c>
+      <c r="I279">
+        <v>422</v>
+      </c>
+      <c r="J279">
+        <v>0</v>
+      </c>
+      <c r="K279" t="s">
+        <v>144</v>
+      </c>
+      <c r="L279" t="s">
+        <v>21</v>
+      </c>
+      <c r="M279" t="s">
+        <v>61</v>
+      </c>
+      <c r="N279" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="280" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A280" t="s">
+        <v>454</v>
+      </c>
+      <c r="B280" t="s">
+        <v>455</v>
+      </c>
+      <c r="C280" t="s">
+        <v>16</v>
+      </c>
+      <c r="D280" t="s">
+        <v>22</v>
+      </c>
+      <c r="F280" t="s">
+        <v>23</v>
+      </c>
+      <c r="G280" t="s">
+        <v>435</v>
+      </c>
+      <c r="H280" t="s">
+        <v>456</v>
+      </c>
+      <c r="I280">
+        <v>3174</v>
+      </c>
+      <c r="J280">
+        <v>0</v>
+      </c>
+      <c r="K280" t="s">
+        <v>20</v>
+      </c>
+      <c r="L280" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="281" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A281" t="s">
+        <v>454</v>
+      </c>
+      <c r="B281" t="s">
+        <v>455</v>
+      </c>
+      <c r="C281" t="s">
+        <v>106</v>
+      </c>
+      <c r="D281" t="s">
+        <v>107</v>
+      </c>
+      <c r="F281" t="s">
+        <v>18</v>
+      </c>
+      <c r="G281" t="s">
+        <v>457</v>
+      </c>
+      <c r="H281" t="s">
+        <v>435</v>
+      </c>
+      <c r="I281">
+        <v>3174</v>
+      </c>
+      <c r="J281">
+        <v>0</v>
+      </c>
+      <c r="K281" t="s">
+        <v>20</v>
+      </c>
+      <c r="L281" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="282" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A282" t="s">
+        <v>454</v>
+      </c>
+      <c r="B282" t="s">
+        <v>455</v>
+      </c>
+      <c r="C282" t="s">
+        <v>106</v>
+      </c>
+      <c r="D282" t="s">
+        <v>31</v>
+      </c>
+      <c r="F282" t="s">
+        <v>18</v>
+      </c>
+      <c r="G282" t="s">
+        <v>458</v>
+      </c>
+      <c r="H282" t="s">
+        <v>435</v>
+      </c>
+      <c r="I282">
+        <v>3174</v>
+      </c>
+      <c r="J282">
+        <v>0</v>
+      </c>
+      <c r="K282" t="s">
+        <v>20</v>
+      </c>
+      <c r="L282" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="283" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A283" t="s">
+        <v>454</v>
+      </c>
+      <c r="B283" t="s">
+        <v>455</v>
+      </c>
+      <c r="C283" t="s">
+        <v>25</v>
+      </c>
+      <c r="D283" t="s">
+        <v>104</v>
+      </c>
+      <c r="F283" t="s">
+        <v>18</v>
+      </c>
+      <c r="G283" t="s">
+        <v>459</v>
+      </c>
+      <c r="H283" t="s">
+        <v>435</v>
+      </c>
+      <c r="I283">
+        <v>3174</v>
+      </c>
+      <c r="J283">
+        <v>0</v>
+      </c>
+      <c r="K283" t="s">
+        <v>20</v>
+      </c>
+      <c r="L283" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="284" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A284" t="s">
+        <v>454</v>
+      </c>
+      <c r="B284" t="s">
+        <v>455</v>
+      </c>
+      <c r="C284" t="s">
+        <v>106</v>
+      </c>
+      <c r="D284" t="s">
+        <v>441</v>
+      </c>
+      <c r="F284" t="s">
+        <v>18</v>
+      </c>
+      <c r="G284" t="s">
+        <v>460</v>
+      </c>
+      <c r="H284" t="s">
+        <v>435</v>
+      </c>
+      <c r="I284">
+        <v>3174</v>
+      </c>
+      <c r="J284">
+        <v>0</v>
+      </c>
+      <c r="K284" t="s">
+        <v>20</v>
+      </c>
+      <c r="L284" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="285" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A285" t="s">
+        <v>454</v>
+      </c>
+      <c r="B285" t="s">
+        <v>455</v>
+      </c>
+      <c r="C285" t="s">
+        <v>56</v>
+      </c>
+      <c r="D285" t="s">
+        <v>461</v>
+      </c>
+      <c r="E285" t="s">
+        <v>444</v>
+      </c>
+      <c r="F285" t="s">
+        <v>35</v>
+      </c>
+      <c r="G285" t="s">
+        <v>435</v>
+      </c>
+      <c r="H285" t="s">
+        <v>462</v>
+      </c>
+      <c r="I285">
+        <v>934</v>
+      </c>
+      <c r="J285">
+        <v>2240</v>
+      </c>
+      <c r="K285" t="s">
+        <v>20</v>
+      </c>
+      <c r="L285" t="s">
+        <v>60</v>
+      </c>
+      <c r="M285" t="s">
+        <v>61</v>
+      </c>
+      <c r="N285" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="286" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>454</v>
+      </c>
+      <c r="B286" t="s">
+        <v>455</v>
+      </c>
+      <c r="C286" t="s">
+        <v>56</v>
+      </c>
+      <c r="D286" t="s">
+        <v>463</v>
+      </c>
+      <c r="E286" t="s">
+        <v>444</v>
+      </c>
+      <c r="F286" t="s">
+        <v>35</v>
+      </c>
+      <c r="G286" t="s">
+        <v>435</v>
+      </c>
+      <c r="H286" t="s">
+        <v>464</v>
+      </c>
+      <c r="I286">
+        <v>3167</v>
+      </c>
+      <c r="J286">
+        <v>7</v>
+      </c>
+      <c r="K286" t="s">
+        <v>20</v>
+      </c>
+      <c r="L286" t="s">
+        <v>21</v>
+      </c>
+      <c r="M286" t="s">
+        <v>61</v>
+      </c>
+      <c r="N286" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="287" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>454</v>
+      </c>
+      <c r="B287" t="s">
+        <v>455</v>
+      </c>
+      <c r="C287" t="s">
+        <v>120</v>
+      </c>
+      <c r="D287" t="s">
+        <v>448</v>
+      </c>
+      <c r="E287" t="s">
+        <v>444</v>
+      </c>
+      <c r="F287" t="s">
+        <v>35</v>
+      </c>
+      <c r="G287" t="s">
+        <v>435</v>
+      </c>
+      <c r="H287" t="s">
+        <v>465</v>
+      </c>
+      <c r="I287">
+        <v>3159</v>
+      </c>
+      <c r="J287">
+        <v>15</v>
+      </c>
+      <c r="K287" t="s">
+        <v>20</v>
+      </c>
+      <c r="L287" t="s">
+        <v>21</v>
+      </c>
+      <c r="M287" t="s">
+        <v>61</v>
+      </c>
+      <c r="N287" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="288" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>454</v>
+      </c>
+      <c r="B288" t="s">
+        <v>455</v>
+      </c>
+      <c r="C288" t="s">
+        <v>120</v>
+      </c>
+      <c r="D288" t="s">
+        <v>450</v>
+      </c>
+      <c r="E288" t="s">
+        <v>444</v>
+      </c>
+      <c r="F288" t="s">
+        <v>35</v>
+      </c>
+      <c r="G288" t="s">
+        <v>435</v>
+      </c>
+      <c r="H288" t="s">
+        <v>466</v>
+      </c>
+      <c r="I288">
+        <v>3147</v>
+      </c>
+      <c r="J288">
+        <v>27</v>
+      </c>
+      <c r="K288" t="s">
+        <v>20</v>
+      </c>
+      <c r="L288" t="s">
+        <v>21</v>
+      </c>
+      <c r="M288" t="s">
+        <v>61</v>
+      </c>
+      <c r="N288" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B303" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C303" t="s">
         <v>16</v>
@@ -11553,10 +12382,10 @@
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B304" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C304" t="s">
         <v>28</v>
@@ -11567,593 +12396,594 @@
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B305" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C305" t="s">
         <v>33</v>
       </c>
       <c r="D305" t="s">
-        <v>436</v>
+        <v>469</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B306" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C306" t="s">
         <v>66</v>
       </c>
       <c r="D306" t="s">
-        <v>437</v>
+        <v>470</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B307" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C307" t="s">
         <v>66</v>
       </c>
       <c r="D307" t="s">
-        <v>438</v>
+        <v>471</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B308" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C308" t="s">
         <v>66</v>
       </c>
       <c r="D308" t="s">
-        <v>439</v>
+        <v>472</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B309" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C309" t="s">
         <v>159</v>
       </c>
       <c r="D309" t="s">
-        <v>440</v>
+        <v>473</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B310" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C310" t="s">
         <v>106</v>
       </c>
       <c r="D310" t="s">
-        <v>441</v>
+        <v>474</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B311" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C311" t="s">
         <v>66</v>
       </c>
       <c r="D311" t="s">
-        <v>442</v>
+        <v>475</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B312" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C312" t="s">
         <v>66</v>
       </c>
       <c r="D312" t="s">
-        <v>443</v>
+        <v>476</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B313" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C313" t="s">
         <v>159</v>
       </c>
       <c r="D313" t="s">
-        <v>444</v>
+        <v>477</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B314" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C314" t="s">
         <v>56</v>
       </c>
       <c r="D314" t="s">
-        <v>445</v>
+        <v>478</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B315" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C315" t="s">
         <v>56</v>
       </c>
       <c r="D315" t="s">
-        <v>446</v>
+        <v>479</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B316" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C316" t="s">
         <v>56</v>
       </c>
       <c r="D316" t="s">
-        <v>447</v>
+        <v>480</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B317" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C317" t="s">
         <v>120</v>
       </c>
       <c r="D317" t="s">
-        <v>448</v>
+        <v>481</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B318" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C318" t="s">
         <v>120</v>
       </c>
       <c r="D318" t="s">
-        <v>449</v>
+        <v>482</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B319" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C319" t="s">
         <v>52</v>
       </c>
       <c r="D319" t="s">
-        <v>450</v>
+        <v>483</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B320" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C320" t="s">
         <v>66</v>
       </c>
       <c r="D320" t="s">
-        <v>451</v>
+        <v>484</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B321" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C321" t="s">
         <v>75</v>
       </c>
       <c r="D321" t="s">
-        <v>452</v>
+        <v>485</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B322" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C322" t="s">
         <v>33</v>
       </c>
       <c r="D322" t="s">
-        <v>453</v>
+        <v>486</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B323" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C323" t="s">
         <v>37</v>
       </c>
       <c r="D323" t="s">
-        <v>454</v>
+        <v>487</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B324" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C324" t="s">
         <v>106</v>
       </c>
       <c r="D324" t="s">
-        <v>455</v>
+        <v>488</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B325" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C325" t="s">
         <v>49</v>
       </c>
       <c r="D325" t="s">
-        <v>456</v>
+        <v>489</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B326" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C326" t="s">
         <v>66</v>
       </c>
       <c r="D326" t="s">
-        <v>457</v>
+        <v>490</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B327" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C327" t="s">
         <v>66</v>
       </c>
       <c r="D327" t="s">
-        <v>458</v>
+        <v>491</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B328" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C328" t="s">
         <v>106</v>
       </c>
       <c r="D328" t="s">
-        <v>459</v>
+        <v>492</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B329" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C329" t="s">
         <v>106</v>
       </c>
       <c r="D329" t="s">
-        <v>460</v>
+        <v>493</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B330" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C330" t="s">
         <v>82</v>
       </c>
       <c r="D330" t="s">
-        <v>461</v>
+        <v>494</v>
       </c>
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B331" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C331" t="s">
         <v>82</v>
       </c>
       <c r="D331" t="s">
-        <v>462</v>
+        <v>495</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B332" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C332" t="s">
         <v>82</v>
       </c>
       <c r="D332" t="s">
-        <v>463</v>
+        <v>496</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B333" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C333" t="s">
         <v>82</v>
       </c>
       <c r="D333" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B334" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C334" t="s">
         <v>66</v>
       </c>
       <c r="D334" t="s">
-        <v>465</v>
+        <v>498</v>
       </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B335" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C335" t="s">
         <v>66</v>
       </c>
       <c r="D335" t="s">
-        <v>466</v>
+        <v>499</v>
       </c>
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B336" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C336" t="s">
         <v>106</v>
       </c>
       <c r="D336" t="s">
-        <v>467</v>
+        <v>500</v>
       </c>
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B337" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C337" t="s">
         <v>106</v>
       </c>
       <c r="D337" t="s">
-        <v>468</v>
+        <v>501</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B338" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C338" t="s">
         <v>159</v>
       </c>
       <c r="D338" t="s">
-        <v>469</v>
+        <v>502</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B339" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C339" t="s">
         <v>56</v>
       </c>
       <c r="D339" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B340" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C340" t="s">
         <v>56</v>
       </c>
       <c r="D340" t="s">
-        <v>471</v>
+        <v>504</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B341" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C341" t="s">
         <v>56</v>
       </c>
       <c r="D341" t="s">
-        <v>472</v>
+        <v>505</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B342" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C342" t="s">
         <v>56</v>
       </c>
       <c r="D342" t="s">
-        <v>473</v>
+        <v>506</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B343" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C343" t="s">
         <v>56</v>
       </c>
       <c r="D343" t="s">
-        <v>474</v>
+        <v>507</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B344" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C344" t="s">
         <v>44</v>
       </c>
       <c r="D344" t="s">
-        <v>475</v>
+        <v>508</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B345" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C345" t="s">
         <v>33</v>
       </c>
       <c r="D345" t="s">
-        <v>476</v>
+        <v>509</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
-        <v>434</v>
+        <v>467</v>
       </c>
       <c r="B346" t="s">
-        <v>435</v>
+        <v>468</v>
       </c>
       <c r="C346" t="s">
         <v>28</v>
       </c>
       <c r="D346" t="s">
-        <v>477</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>